<commit_message>
chore: remove embedded scrapling repo from index && add isTrust Signal in level 1
</commit_message>
<xml_diff>
--- a/automation/anti-detect框架整理.xlsx
+++ b/automation/anti-detect框架整理.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>Name</t>
   </si>
@@ -39,6 +39,9 @@
   </si>
   <si>
     <t>timestamp</t>
+  </si>
+  <si>
+    <t>result</t>
   </si>
   <si>
     <t>Puppeteer-extra-stealth</t>
@@ -106,6 +109,9 @@
     <t>https://github.com/Kaliiiiiiiiii-Vinyzu/patchright-python</t>
   </si>
   <si>
+    <t>2026/3/4 16:46:06、2026/3/16 10:39:39</t>
+  </si>
+  <si>
     <t>Camoufox</t>
   </si>
   <si>
@@ -144,6 +150,12 @@
     <t>https://github.com/daijro/camoufox</t>
   </si>
   <si>
+    <t>2026/3/6 1:50:00、2026/3/13/ 19:33:56</t>
+  </si>
+  <si>
+    <t>❌</t>
+  </si>
+  <si>
     <t>SeleniumBase</t>
   </si>
   <si>
@@ -153,6 +165,9 @@
     <t>https://github.com/seleniumbase/SeleniumBase</t>
   </si>
   <si>
+    <t>2026/3/3 20:12:09、2026/3/16 10:25:00</t>
+  </si>
+  <si>
     <t>Rebrowser Playwright</t>
   </si>
   <si>
@@ -162,6 +177,9 @@
     <t>https://github.com/rebrowser/rebrowser-playwright</t>
   </si>
   <si>
+    <t>没测试，工具原理同下</t>
+  </si>
+  <si>
     <t>Rebrowser Puppeteer</t>
   </si>
   <si>
@@ -171,6 +189,9 @@
     <t>https://github.com/rebrowser/rebrowser-puppeteer</t>
   </si>
   <si>
+    <t>2026/3/6 19:48:46、2026/3/16 10:48:00</t>
+  </si>
+  <si>
     <t>Puppeteer Real Browser</t>
   </si>
   <si>
@@ -187,6 +208,30 @@
   </si>
   <si>
     <t>https://github.com/MiddleSchoolStudent/BotBrowser</t>
+  </si>
+  <si>
+    <t>脚本需要money</t>
+  </si>
+  <si>
+    <t>GeekezBrowser</t>
+  </si>
+  <si>
+    <t>GeekEZ Browser is a professional anti-detect browser built on Electron and Puppeteer, integrated with the powerful Xray-core.</t>
+  </si>
+  <si>
+    <t>https://github.com/EchoHS/GeekezBrowser</t>
+  </si>
+  <si>
+    <t>scrapling</t>
+  </si>
+  <si>
+    <t>agent-broswer</t>
+  </si>
+  <si>
+    <t>agent+chromium</t>
+  </si>
+  <si>
+    <t>llm_srcaper</t>
   </si>
 </sst>
 </file>
@@ -844,20 +889,26 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="6" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1385,16 +1436,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="3"/>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="47.75" customWidth="1"/>
     <col min="2" max="2" width="101.759615384615" customWidth="1"/>
     <col min="3" max="3" width="79.9615384615385" customWidth="1"/>
-    <col min="4" max="4" width="15.3846153846154" customWidth="1"/>
+    <col min="4" max="4" width="39.3846153846154" customWidth="1"/>
+    <col min="5" max="5" width="24.8461538461538" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1404,137 +1456,207 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" ht="32" spans="1:4">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="s">
+    <row r="2" ht="32" spans="1:5">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="4">
+      <c r="C2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="5">
         <v>46084.8222453704</v>
       </c>
+      <c r="E2" s="2"/>
     </row>
-    <row r="3" ht="32" spans="1:4">
-      <c r="A3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="3" ht="32" spans="1:5">
+      <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="4"/>
+      <c r="C3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="5">
+        <v>46097.4310416667</v>
+      </c>
+      <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    <row r="4" spans="1:5">
+      <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="C4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="5">
+        <v>46097.4629166667</v>
+      </c>
+      <c r="E4" s="2"/>
     </row>
-    <row r="5" ht="32" spans="1:4">
-      <c r="A5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="2" t="s">
+    <row r="5" ht="32" spans="1:5">
+      <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="4">
-        <v>46085.6986805556</v>
-      </c>
+      <c r="C5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="2"/>
     </row>
-    <row r="6" ht="32" spans="1:4">
-      <c r="A6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="3" t="s">
+    <row r="6" ht="32" spans="1:5">
+      <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="4">
-        <v>46087.0763888889</v>
+      <c r="B6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="7" ht="32" spans="1:4">
-      <c r="A7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="4">
-        <v>46084.8417708333</v>
-      </c>
+    <row r="7" ht="32" spans="1:5">
+      <c r="A7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="2"/>
     </row>
-    <row r="8" ht="32" spans="1:3">
-      <c r="A8" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>24</v>
+    <row r="8" ht="32" spans="1:5">
+      <c r="A8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
-    <row r="9" ht="32" spans="1:4">
-      <c r="A9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="4">
-        <v>46087.8255324074</v>
-      </c>
+    <row r="9" ht="32" spans="1:5">
+      <c r="A9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="2"/>
     </row>
-    <row r="10" ht="32" spans="1:3">
-      <c r="A10" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>30</v>
-      </c>
+    <row r="10" ht="32" spans="1:5">
+      <c r="A10" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="5">
+        <v>46097.4693402778</v>
+      </c>
+      <c r="E10" s="2"/>
     </row>
-    <row r="11" ht="32" spans="1:4">
-      <c r="A11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" s="4">
+    <row r="11" ht="32" spans="1:5">
+      <c r="A11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="5">
         <v>46087.9449305556</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="5">
+        <v>46090.7950115741</v>
+      </c>
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="5">
+        <v>46097.6972337963</v>
+      </c>
+      <c r="E13" s="2"/>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1547,8 +1669,9 @@
     <hyperlink ref="C7" r:id="rId6" display="https://github.com/seleniumbase/SeleniumBase" tooltip="https://github.com/seleniumbase/SeleniumBase?ref=blog.castle.io"/>
     <hyperlink ref="C8" r:id="rId7" display="https://github.com/rebrowser/rebrowser-playwright" tooltip="https://github.com/rebrowser/rebrowser-playwright?ref=blog.castle.io"/>
     <hyperlink ref="C9" r:id="rId8" display="https://github.com/rebrowser/rebrowser-puppeteer" tooltip="https://github.com/rebrowser/rebrowser-puppeteer?ref=blog.castle.io"/>
-    <hyperlink ref="C10" r:id="rId9" display="https://github.com/ZFC-Digital/puppeteer-real-browser" tooltip="https://github.com/ZFC-Digital/puppeteer-real-browser?ref=blog.castle.io"/>
+    <hyperlink ref="C10" r:id="rId9" display="https://github.com/ZFC-Digital/puppeteer-real-browser" tooltip="https://github.com/ZFC-Digital/puppeteer-real-browser"/>
     <hyperlink ref="C11" r:id="rId10" display="https://github.com/MiddleSchoolStudent/BotBrowser" tooltip="https://github.com/MiddleSchoolStudent/BotBrowser?ref=blog.castle.io"/>
+    <hyperlink ref="C12" r:id="rId11" display="https://github.com/EchoHS/GeekezBrowser"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>